<commit_message>
Upgrade: Implement probabilistic simulation modeling demand and lead time volatility
</commit_message>
<xml_diff>
--- a/input_template.xlsx
+++ b/input_template.xlsx
@@ -727,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -737,6 +737,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -775,6 +776,11 @@
           <t>Lead_Time_Days</t>
         </is>
       </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Lead_Time_StdDev_Days</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -806,6 +812,9 @@
       <c r="G2" s="9" t="n">
         <v>7</v>
       </c>
+      <c r="H2" s="9" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -837,6 +846,9 @@
       <c r="G3" s="13" t="n">
         <v>10</v>
       </c>
+      <c r="H3" s="13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -868,6 +880,9 @@
       <c r="G4" s="9" t="n">
         <v>12</v>
       </c>
+      <c r="H4" s="9" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -899,6 +914,9 @@
       <c r="G5" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="H5" s="13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -929,6 +947,9 @@
       </c>
       <c r="G6" s="9" t="n">
         <v>6</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>
@@ -943,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -952,6 +973,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -985,6 +1007,11 @@
           <t>Reorder_Quantity_Units</t>
         </is>
       </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Demand_StdDev_Units</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1009,6 +1036,9 @@
       <c r="F2" s="9" t="n">
         <v>150</v>
       </c>
+      <c r="G2" s="9" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -1033,6 +1063,9 @@
       <c r="F3" s="13" t="n">
         <v>100</v>
       </c>
+      <c r="G3" s="13" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1057,6 +1090,9 @@
       <c r="F4" s="9" t="n">
         <v>120</v>
       </c>
+      <c r="G4" s="9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1081,6 +1117,9 @@
       <c r="F5" s="13" t="n">
         <v>100</v>
       </c>
+      <c r="G5" s="13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1105,6 +1144,9 @@
       <c r="F6" s="9" t="n">
         <v>80</v>
       </c>
+      <c r="G6" s="9" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1128,6 +1170,9 @@
       </c>
       <c r="F7" s="13" t="n">
         <v>150</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Execution Run: Update template and OOS analysis report for June 2026 dates
</commit_message>
<xml_diff>
--- a/input_template.xlsx
+++ b/input_template.xlsx
@@ -1245,7 +1245,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D2" s="14" t="n">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D3" s="15" t="n">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D4" s="14" t="n">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D5" s="15" t="n">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D6" s="14" t="n">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D7" s="15" t="n">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="D8" s="14" t="n">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="D9" s="15" t="n">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="D10" s="14" t="n">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="D11" s="15" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="D12" s="14" t="n">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="D13" s="15" t="n">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D14" s="14" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D16" s="14" t="n">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D18" s="14" t="n">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D20" s="14" t="n">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D22" s="14" t="n">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D24" s="14" t="n">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D26" s="14" t="n">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D28" s="14" t="n">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D30" s="14" t="n">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D31" s="15" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D32" s="14" t="n">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D33" s="15" t="n">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D34" s="14" t="n">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D35" s="15" t="n">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D36" s="14" t="n">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D37" s="15" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D38" s="14" t="n">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D39" s="15" t="n">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D40" s="14" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D41" s="15" t="n">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D42" s="14" t="n">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D43" s="15" t="n">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D44" s="14" t="n">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D45" s="15" t="n">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D46" s="14" t="n">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D47" s="15" t="n">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D48" s="14" t="n">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D49" s="15" t="n">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D50" s="14" t="n">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D51" s="15" t="n">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D52" s="14" t="n">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D53" s="15" t="n">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D54" s="14" t="n">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D55" s="15" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D56" s="14" t="n">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D57" s="15" t="n">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D58" s="14" t="n">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D59" s="15" t="n">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D60" s="14" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D61" s="15" t="n">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D62" s="14" t="n">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D63" s="15" t="n">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D64" s="14" t="n">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D65" s="15" t="n">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D66" s="14" t="n">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D67" s="15" t="n">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D68" s="14" t="n">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D69" s="15" t="n">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D70" s="14" t="n">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D71" s="15" t="n">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D72" s="14" t="n">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D73" s="15" t="n">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">

</xml_diff>